<commit_message>
added coop event ui
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/Coop.xlsx
+++ b/Assets/StreamingAssets/Configurations/Coop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1687C12-2C51-426F-B3AD-1E2950BBE29D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26089D1B-0756-4F35-831A-E192745A1168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" xr2:uid="{85C794E5-BD16-4817-A60E-1226C928BE3E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{85C794E5-BD16-4817-A60E-1226C928BE3E}"/>
   </bookViews>
   <sheets>
     <sheet name="CoopEvents" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -42,9 +42,6 @@
     <t>EventTypes</t>
   </si>
   <si>
-    <t>Effects</t>
-  </si>
-  <si>
     <t>UnlockLevel</t>
   </si>
   <si>
@@ -55,6 +52,30 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>Recovery</t>
+  </si>
+  <si>
+    <t>Effect1</t>
+  </si>
+  <si>
+    <t>E1Param</t>
+  </si>
+  <si>
+    <t>Effect2</t>
+  </si>
+  <si>
+    <t>E2Param</t>
+  </si>
+  <si>
+    <t>Effect3</t>
+  </si>
+  <si>
+    <t>E3Param</t>
+  </si>
+  <si>
+    <t>Stream,Practice</t>
   </si>
 </sst>
 </file>
@@ -78,9 +99,18 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFF0000"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -90,8 +120,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,36 +437,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{094FDAA9-F479-41E4-9B48-92DE073E19D4}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="25.42578125" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
       <c r="D1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>2</v>
+      </c>
+      <c r="D2">
+        <v>0.5</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>0.7</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>